<commit_message>
feat: expand sample target repo demo data
</commit_message>
<xml_diff>
--- a/sample_data/sample_developers.xlsx
+++ b/sample_data/sample_developers.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,189 +458,162 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DEV_DARKBO0</t>
+          <t>DEV_MINSU_KIM</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ByoungHyeon</t>
+          <t>김민수</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>darkbo0@kakao.com</t>
+          <t>minsu.kim@sample.local</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Frontend Developer</t>
+          <t>개발자</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Spring MVC Controller, Thymeleaf/HTML, CSS, SCSS</t>
+          <t>주문 업무, Spring MVC, JSP, MyBatis</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DEV_CHERO77</t>
+          <t>DEV_JIHOON_PARK</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ino5</t>
+          <t>박지훈</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>chero77@naver.com</t>
+          <t>jihoon.park@sample.local</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Frontend Developer</t>
+          <t>개발자</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Spring MVC Controller, Service Layer, Repository/JPA, Thymeleaf/HTML, JavaScript</t>
+          <t>재고/매출 업무, Spring MVC, JSP, MyBatis</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DEV_KAILYYY02</t>
+          <t>DEV_SEHUN_OH</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>kaily22</t>
+          <t>오세훈</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>kailyyy02@gmail.com</t>
+          <t>sehun.oh@sample.local</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Frontend Developer</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Spring MVC Controller, Service Layer, Repository/JPA, Thymeleaf/HTML, JavaScript</t>
+          <t>요구사항 분석, 설계 검토, 개발 리딩</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DEV_HANNAGOOD0805</t>
+          <t>DEV_JIEUN_LEE</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>leehanna0805</t>
+          <t>이지은</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>hannagood0805@gmail.com</t>
+          <t>jieun.lee@sample.local</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Frontend Developer</t>
+          <t>개발자</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Spring MVC Controller, Service Layer, Repository/JPA, Thymeleaf/HTML, JavaScript</t>
+          <t>결제/대시보드 업무, Spring MVC, JSP, MyBatis</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DEV_58283314_SUYEONCHOI7807</t>
+          <t>DEV_SEOYEON_JUNG</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>suyeon</t>
+          <t>정서연</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>58283314+suyeonChoi7807@users.noreply.github.com</t>
+          <t>seoyeon.jung@sample.local</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Technical Writer</t>
+          <t>QA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>테스트 케이스, 결함 관리, 검수 지원</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DEV_SUYEON2205</t>
+          <t>DEV_HYUNWOO_CHOI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>suyeonChoi7807</t>
+          <t>최현우</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>suyeon2205@naver.com</t>
+          <t>hyunwoo.choi@sample.local</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Frontend Developer</t>
+          <t>PM</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Spring MVC Controller, Service Layer, Repository/JPA, Thymeleaf/HTML, JavaScript</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>DEV_GUSQHDUD96</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>영보</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>gusqhdud96@gmail.com</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Technical Writer</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Thymeleaf/HTML, Documentation</t>
+          <t>사업관리, 일정관리, 고객 협의</t>
         </is>
       </c>
     </row>

</xml_diff>